<commit_message>
feat: implement 6 perubahan JURNALKU
- Absensi siswa: pisah masuk/pulang + jam masuk/pulang
- Catatan Kepribadian: sederhanakan jadi Sikap Umum + Catatan Wali Kelas
- Admin/operator/TU/kepala: menu Ceklok Saya
- Rekap absensi: mode weekly/monthly/semester/yearly
- Jurnal mengajar: auto-fill mapel & rombel dari jadwal
- Geolokasi: presisi tinggi + tombol Ambil Lokasi Saya

Backend: migrasi kolom, endpoint baru
Frontend: build sukses, UI updated
</commit_message>
<xml_diff>
--- a/public/templates/template-gtk.xlsx
+++ b/public/templates/template-gtk.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Data GTK" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,21 +397,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:O3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="5.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
     <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" customWidth="1"/>
-    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="3.83203125" customWidth="1"/>
+    <col min="15" max="15" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,6 +461,12 @@
       <c r="M2" t="str">
         <v>Email</v>
       </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v>PERHATIAN</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -500,13 +508,16 @@
       <c r="M3" t="str">
         <v>guru@contoh.sch.id</v>
       </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v>JK: L/P. TGL Lahir: YYYY-MM-DD. Status Kepegawaian: PNS/PPPK/GTY/Honorer.</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
-  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>